<commit_message>
Tinggal ubah ke bahasa Arab
</commit_message>
<xml_diff>
--- a/Mufrodat/September 2025/mufrodat.xlsx
+++ b/Mufrodat/September 2025/mufrodat.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ASATIDZ\Zen\bahasa-terbaru\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\bahasa-terbaru\Mufrodat\September 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B3C17C-D6C6-449F-8962-35855993AFE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9579EA16-29C7-416D-A788-43BB0F507583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mufrodat" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="103">
   <si>
     <t>Nomor</t>
   </si>
@@ -50,279 +50,6 @@
     <t>Bahasa Indonesia</t>
   </si>
   <si>
-    <t>Bahasa Arab</t>
-  </si>
-  <si>
-    <t>Jangan tidur di shaff depan</t>
-  </si>
-  <si>
-    <t>Kelas tiga di shaff pertama</t>
-  </si>
-  <si>
-    <t>Jangan main lari-lari</t>
-  </si>
-  <si>
-    <t>Ambilkan Quranku dong</t>
-  </si>
-  <si>
-    <t>Sudah shalat sunnah belum?</t>
-  </si>
-  <si>
-    <t>Jangan berisik di masjid</t>
-  </si>
-  <si>
-    <t>Jangan salto, nanti roboh</t>
-  </si>
-  <si>
-    <t>Kerja bagus</t>
-  </si>
-  <si>
-    <t>Ada buaya</t>
-  </si>
-  <si>
-    <t>Ada duit kah?</t>
-  </si>
-  <si>
-    <t>Izin dulu</t>
-  </si>
-  <si>
-    <t>Pergi ke tambang yuk</t>
-  </si>
-  <si>
-    <t>Tolong ambilkan parfum</t>
-  </si>
-  <si>
-    <t>Ngelunjak kali kau</t>
-  </si>
-  <si>
-    <t>Tolong belikan es</t>
-  </si>
-  <si>
-    <t>Bersihin, kotor nih</t>
-  </si>
-  <si>
-    <t>Sapu lantainya</t>
-  </si>
-  <si>
-    <t>Mana kopiahku?</t>
-  </si>
-  <si>
-    <t>Nyalakan kipasnya</t>
-  </si>
-  <si>
-    <t>Wih, ngerinya pang</t>
-  </si>
-  <si>
-    <t>Nggak ngotak bah</t>
-  </si>
-  <si>
-    <t>Jangan shake es, takut tumpah</t>
-  </si>
-  <si>
-    <t>Nggak boleh mainan di kamar mandi</t>
-  </si>
-  <si>
-    <t>Kamu sakit kah?</t>
-  </si>
-  <si>
-    <t>Santai dong mukanya</t>
-  </si>
-  <si>
-    <t>Berapa menit lagi adzan?</t>
-  </si>
-  <si>
-    <t>Wudhu sebelum shalat!</t>
-  </si>
-  <si>
-    <t>Sana jauh-jauh</t>
-  </si>
-  <si>
-    <t>Mana tongkat mimbar</t>
-  </si>
-  <si>
-    <t>Mic mati</t>
-  </si>
-  <si>
-    <t>Sajadah rusak</t>
-  </si>
-  <si>
-    <t>Vacum ambal</t>
-  </si>
-  <si>
-    <t>Piket masjid</t>
-  </si>
-  <si>
-    <t>Hijab jatuh</t>
-  </si>
-  <si>
-    <t>Hayooo mimbar rusak</t>
-  </si>
-  <si>
-    <t>Hayooo sajadah robek</t>
-  </si>
-  <si>
-    <t>Pakai sarung</t>
-  </si>
-  <si>
-    <t>Rapiin Quran</t>
-  </si>
-  <si>
-    <t>Nggak boleh ngomong kasar</t>
-  </si>
-  <si>
-    <t>Eh, aku mau cerita sama kalian</t>
-  </si>
-  <si>
-    <t>Ambilkan minum nah</t>
-  </si>
-  <si>
-    <t>Jangan lari-lari</t>
-  </si>
-  <si>
-    <t>Isi shaffnya</t>
-  </si>
-  <si>
-    <t>Siapa yang adzan?</t>
-  </si>
-  <si>
-    <t>Jangan freestyle di masjid. Nanti roboh</t>
-  </si>
-  <si>
-    <t>لَا تَنَمْ فِي الصَّفِّ الْأَمَامِيِّ</t>
-  </si>
-  <si>
-    <t>ٱلْمَرْحَلَةُ ٱلثَّالِثَةُ فِي ٱلصَّفِّ ٱلْأَوَّلِ</t>
-  </si>
-  <si>
-    <t>لَا تَلْعَبْ بِالْجَرْيِ</t>
-  </si>
-  <si>
-    <t>هَاتِ لِي قُرْآنِي</t>
-  </si>
-  <si>
-    <t>هَلْ صَلَّيْتَ السُّنَّةَ؟</t>
-  </si>
-  <si>
-    <t>لَا تُزْعِجْ فِي الْمَسْجِدِ</t>
-  </si>
-  <si>
-    <t>لَا تَقُمْ بِالسَّلْتُو، قَدْ يَسْقُطَ</t>
-  </si>
-  <si>
-    <t>عَمَلٌ جَيِّدٌ</t>
-  </si>
-  <si>
-    <t>هُنَاكَ تِمْسَاحٌ!</t>
-  </si>
-  <si>
-    <t>هَلْ عِنْدَكَ فُلُوس؟</t>
-  </si>
-  <si>
-    <t>اسْتَأْذِنْ أَوَّلًا</t>
-  </si>
-  <si>
-    <t>هَيَّا نَذْهَبْ إِلَى الْمَنْجَمِ</t>
-  </si>
-  <si>
-    <t>مِنْ فَضْلِكَ، أَحْضِرْ لِيَ الْعِطْرَ</t>
-  </si>
-  <si>
-    <t>أَنْتَ وَقِحٌ جِدًّا!</t>
-  </si>
-  <si>
-    <t>مِنْ فَضْلِكَ، اشْتَرِ لِيَ ثَلْجًا</t>
-  </si>
-  <si>
-    <t>نَظِّفْ، إِنَّهُ مُتَّسِخٌ</t>
-  </si>
-  <si>
-    <t>اكْنُسِ الْأَرْضَ</t>
-  </si>
-  <si>
-    <t>أَيْنَ قَلَنْسُوَتِي؟</t>
-  </si>
-  <si>
-    <t>شَغِّلِ الْمِرْوَحَةَ</t>
-  </si>
-  <si>
-    <t>وَاه! إِنَّهُ مُخِيفٌ جِدًّا!</t>
-  </si>
-  <si>
-    <t>هٰذَا غَيْرُ مَعْقُولٍ!</t>
-  </si>
-  <si>
-    <t>لَا تَهُزَّ الثَّلْجَ، قَدْ يَنْسَكِبَ</t>
-  </si>
-  <si>
-    <t>لَا يَجُوزُ اللَّعِبُ فِي الْحَمَّامِ</t>
-  </si>
-  <si>
-    <t>هَلْ أَنْتَ مَرِيضٌ؟</t>
-  </si>
-  <si>
-    <t>هَدِّئْ وَجْهَكَ قَلِيلًا</t>
-  </si>
-  <si>
-    <t>كَمْ بَقِيَ عَلَى الْأَذَانِ؟</t>
-  </si>
-  <si>
-    <t>تَوَضَّأْ قَبْلَ الصَّلَاةِ!</t>
-  </si>
-  <si>
-    <t>ابْتَعِدْ!</t>
-  </si>
-  <si>
-    <t>أَيْنَ عَصَا الْمِنْبَرِ؟</t>
-  </si>
-  <si>
-    <t>الْمِيكْرُوفُونُ مَطْفَأٌ</t>
-  </si>
-  <si>
-    <t>السَّجَّادَةُ مُمَزَّقَةٌ</t>
-  </si>
-  <si>
-    <t>نَظِّفِ الْفُرُشَ بِالْمِكْنَسَةِ الْكَهْرَبَائِيَّةِ</t>
-  </si>
-  <si>
-    <t>نَوْبَةُ النَّظَافَةِ فِي الْمَسْجِدِ</t>
-  </si>
-  <si>
-    <t>السِّتَارَةُ سَقَطَتْ</t>
-  </si>
-  <si>
-    <t>هَيَّهْ! الْمِنْبَرُ مَكْسُورٌ!</t>
-  </si>
-  <si>
-    <t>هَيَّهْ! السَّجَّادَةُ مُمَزَّقَةٌ!</t>
-  </si>
-  <si>
-    <t>ٱلْبَسِ ٱلْإِزَارَ</t>
-  </si>
-  <si>
-    <t>رَتِّبِ الْقُرْآنَ</t>
-  </si>
-  <si>
-    <t>لَا تَتَكَلَّمْ بِكَلِمَاتٍ بَذِيئَةٍ</t>
-  </si>
-  <si>
-    <t>أَهْ، أُرِيدُ أَنْ أُحَدِّثَكُمْ بِقِصَّةٍ</t>
-  </si>
-  <si>
-    <t>أَحْضِرْ لِي شَرَابًا، نَحْ</t>
-  </si>
-  <si>
-    <t>لَا تَجْرِ!</t>
-  </si>
-  <si>
-    <t>أَتْمِمُوا الصَّفَّ</t>
-  </si>
-  <si>
-    <t>مَنْ يُؤَذِّنُ؟</t>
-  </si>
-  <si>
-    <t>لَا تَقُمْ بِالْحَرَكَاتِ الْحُرَّةِ فِي الْمَسْجِدِ، قَدْ يَسْقُطَ</t>
-  </si>
-  <si>
     <t>Ahmad Abdullah Kholis</t>
   </si>
   <si>
@@ -480,6 +207,150 @@
   </si>
   <si>
     <t>Nama</t>
+  </si>
+  <si>
+    <t>Umar Abdurrosyid Assary</t>
+  </si>
+  <si>
+    <t>Bahasa Arab Putra</t>
+  </si>
+  <si>
+    <t>Bahasa Arab Putri</t>
+  </si>
+  <si>
+    <t>Baru, baru</t>
+  </si>
+  <si>
+    <t>Buat kamu</t>
+  </si>
+  <si>
+    <t>Tolong aku</t>
+  </si>
+  <si>
+    <t>Bantuin nah</t>
+  </si>
+  <si>
+    <t>Siapa kamu?</t>
+  </si>
+  <si>
+    <t>Karpetnya wangi sekali</t>
+  </si>
+  <si>
+    <t>Sapu musholahnya</t>
+  </si>
+  <si>
+    <t>Nyalakan semua kipasnya</t>
+  </si>
+  <si>
+    <t>Rapikan sajadahnya</t>
+  </si>
+  <si>
+    <t>Jangan mainin mic</t>
+  </si>
+  <si>
+    <t>Sajadahnya jangan lupa dilipat</t>
+  </si>
+  <si>
+    <t>Sudah pada shalat sunnah kah?</t>
+  </si>
+  <si>
+    <t>Penuhin shaf depan</t>
+  </si>
+  <si>
+    <t>Hei, baca doa dulu sebelum masuk masjid</t>
+  </si>
+  <si>
+    <t>Quranmu mana?</t>
+  </si>
+  <si>
+    <t>Ntaran ajah, aku mau shalat dulu</t>
+  </si>
+  <si>
+    <t>Gelap banget dah mushollahnya</t>
+  </si>
+  <si>
+    <t>Kalau adzan, jangan ribut</t>
+  </si>
+  <si>
+    <t>Kenapa belum siap-siap shalat?</t>
+  </si>
+  <si>
+    <t>Ini masjid, nggak usah banyak tingkah</t>
+  </si>
+  <si>
+    <t>Jangan teriak-teriak saat adzan</t>
+  </si>
+  <si>
+    <t>Sudah tahajud kah?</t>
+  </si>
+  <si>
+    <t>Mana sajadahmu?</t>
+  </si>
+  <si>
+    <t>Masjidnya indah sekali</t>
+  </si>
+  <si>
+    <t>Kamu udah wudhu belum?</t>
+  </si>
+  <si>
+    <t>Sudah qomat nggak sih?</t>
+  </si>
+  <si>
+    <t>Wudhu bareng yuk</t>
+  </si>
+  <si>
+    <t>Bagi-bagi sajadahnya dong</t>
+  </si>
+  <si>
+    <t>Ayo siap-siap sholat</t>
+  </si>
+  <si>
+    <t>Siapa jadi imam?</t>
+  </si>
+  <si>
+    <t>Rapatkan shafnya?</t>
+  </si>
+  <si>
+    <t>Jaga adabnya di masjid</t>
+  </si>
+  <si>
+    <t>Jangan ribut kalau mau shalat</t>
+  </si>
+  <si>
+    <t>Nanti malam kajian di masjid</t>
+  </si>
+  <si>
+    <t>Tadi aku shalat di masjid</t>
+  </si>
+  <si>
+    <t>Di masjid tadi ada kucing</t>
+  </si>
+  <si>
+    <t>Kalau masuk masjid, berdoa ya</t>
+  </si>
+  <si>
+    <t>Cepat rapatin shafnya</t>
+  </si>
+  <si>
+    <t>Sajadah siapa ini?</t>
+  </si>
+  <si>
+    <t>Ayo kita shalat, sudah adzan</t>
+  </si>
+  <si>
+    <t>Adzannya jam berapa?</t>
+  </si>
+  <si>
+    <t>Teras masjidnya kotor</t>
+  </si>
+  <si>
+    <t>Tangganya basah</t>
+  </si>
+  <si>
+    <t>Susun sudah shafnya</t>
+  </si>
+  <si>
+    <t>Siapa ini yang nyapu ruang shalat?</t>
   </si>
 </sst>
 </file>
@@ -884,7 +755,7 @@
   <cols>
     <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -895,7 +766,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>2</v>
+        <v>56</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>57</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -905,47 +779,42 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>48</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11"/>
       <c r="B3" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>49</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
     </row>
     <row r="4" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11"/>
       <c r="B4" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>50</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
     </row>
     <row r="5" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11"/>
       <c r="B5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>51</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>52</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
     </row>
     <row r="7" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
@@ -953,47 +822,42 @@
         <v>2</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>53</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
     </row>
     <row r="8" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12"/>
       <c r="B8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>54</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="12"/>
       <c r="B9" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>55</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
     </row>
     <row r="10" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
       <c r="B10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>56</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
     </row>
     <row r="11" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
       <c r="B11" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>57</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
     </row>
     <row r="12" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
@@ -1001,335 +865,300 @@
         <v>3</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>58</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
     </row>
     <row r="13" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11"/>
       <c r="B13" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>59</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
     </row>
     <row r="14" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
       <c r="B14" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>60</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
     </row>
     <row r="15" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11"/>
       <c r="B15" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>61</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
     </row>
     <row r="16" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11"/>
       <c r="B16" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+    </row>
+    <row r="17" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12">
         <f t="shared" ref="A17" si="1">A12+1</f>
         <v>4</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+    </row>
+    <row r="18" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12"/>
       <c r="B18" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12"/>
       <c r="B19" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+    </row>
+    <row r="20" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12"/>
       <c r="B20" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12"/>
       <c r="B21" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+    </row>
+    <row r="22" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
         <f t="shared" ref="A22" si="2">A17+1</f>
         <v>5</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+    </row>
+    <row r="23" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11"/>
       <c r="B23" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+    </row>
+    <row r="24" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11"/>
       <c r="B24" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+    </row>
+    <row r="25" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
       <c r="B25" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+    </row>
+    <row r="26" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11"/>
       <c r="B26" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+    </row>
+    <row r="27" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="12">
         <f t="shared" ref="A27" si="3">A22+1</f>
         <v>6</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+    </row>
+    <row r="28" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="12"/>
       <c r="B28" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+    </row>
+    <row r="29" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="12"/>
       <c r="B29" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+    </row>
+    <row r="30" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="12"/>
       <c r="B30" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+    </row>
+    <row r="31" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12"/>
       <c r="B31" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+    </row>
+    <row r="32" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11">
         <f t="shared" ref="A32" si="4">A27+1</f>
         <v>7</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+    </row>
+    <row r="33" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11"/>
       <c r="B33" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+    </row>
+    <row r="34" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11"/>
       <c r="B34" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+    </row>
+    <row r="35" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11"/>
       <c r="B35" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+    </row>
+    <row r="36" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11"/>
       <c r="B36" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+    </row>
+    <row r="37" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="12">
         <f t="shared" ref="A37" si="5">A32+1</f>
         <v>8</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+    </row>
+    <row r="38" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+    </row>
+    <row r="39" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="12"/>
       <c r="B39" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+    </row>
+    <row r="40" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="12"/>
       <c r="B40" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+    </row>
+    <row r="41" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="12"/>
       <c r="B41" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+    </row>
+    <row r="42" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11">
         <f t="shared" ref="A42" si="6">A37+1</f>
         <v>9</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+    </row>
+    <row r="43" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="11"/>
       <c r="B43" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="C43" s="5"/>
+      <c r="D43" s="5"/>
+    </row>
+    <row r="44" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="11"/>
       <c r="B44" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+    </row>
+    <row r="45" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="11"/>
       <c r="B45" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+    </row>
+    <row r="46" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="11"/>
       <c r="B46" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>92</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="C46" s="5"/>
+      <c r="D46" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -1354,7 +1183,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
@@ -1367,7 +1196,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>145</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1375,7 +1204,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>93</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1384,7 +1213,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>99</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1393,7 +1222,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>100</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1402,7 +1231,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>101</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1411,7 +1240,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>103</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1420,7 +1249,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>104</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1429,7 +1258,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>105</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1438,7 +1267,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1447,7 +1276,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>108</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1455,7 +1284,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>109</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1463,7 +1292,7 @@
         <v>2</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>110</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1471,7 +1300,7 @@
         <v>3</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1479,7 +1308,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>112</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1487,7 +1316,7 @@
         <v>5</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>113</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1495,7 +1324,7 @@
         <v>6</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>114</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1503,7 +1332,7 @@
         <v>7</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>115</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1511,7 +1340,7 @@
         <v>8</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>117</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1519,7 +1348,7 @@
         <v>9</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>119</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1527,7 +1356,7 @@
         <v>1</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>121</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1535,7 +1364,7 @@
         <v>2</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>122</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1543,7 +1372,7 @@
         <v>3</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>123</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1551,7 +1380,7 @@
         <v>4</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>124</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1559,7 +1388,7 @@
         <v>5</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>125</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1567,7 +1396,7 @@
         <v>6</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>128</v>
+        <v>37</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1575,7 +1404,7 @@
         <v>7</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>129</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1583,7 +1412,7 @@
         <v>8</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>130</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1591,7 +1420,7 @@
         <v>9</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>134</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1599,7 +1428,7 @@
         <v>1</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>138</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1607,7 +1436,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>139</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1615,7 +1444,7 @@
         <v>3</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>140</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1623,7 +1452,15 @@
         <v>4</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>141</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>5</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1651,7 +1488,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>145</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1659,7 +1496,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>94</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1668,7 +1505,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>95</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1677,7 +1514,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>96</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1686,7 +1523,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>97</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1695,7 +1532,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>98</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1704,7 +1541,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1713,7 +1550,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>107</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1722,7 +1559,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1731,7 +1568,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>118</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1739,7 +1576,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>120</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1747,7 +1584,7 @@
         <v>2</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1755,7 +1592,7 @@
         <v>3</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>127</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1763,7 +1600,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>131</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1771,7 +1608,7 @@
         <v>5</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>132</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1779,7 +1616,7 @@
         <v>6</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>133</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1787,7 +1624,7 @@
         <v>7</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>135</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1795,7 +1632,7 @@
         <v>8</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>136</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1803,7 +1640,7 @@
         <v>9</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>137</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1811,7 +1648,7 @@
         <v>1</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>142</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1819,7 +1656,7 @@
         <v>2</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>143</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1827,7 +1664,7 @@
         <v>3</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>144</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>